<commit_message>
full lapso; experiment scripts
</commit_message>
<xml_diff>
--- a/case14.xlsx
+++ b/case14.xlsx
@@ -2285,7 +2285,7 @@
         <v>0</v>
       </c>
       <c r="F18">
-        <v>55.97512868856456</v>
+        <v>55.97512868856458</v>
       </c>
       <c r="G18">
         <v>0</v>
@@ -2408,7 +2408,7 @@
         <v>0</v>
       </c>
       <c r="F21">
-        <v>31.76492603364068</v>
+        <v>31.7649260336407</v>
       </c>
       <c r="G21">
         <v>0</v>

</xml_diff>